<commit_message>
Refactor: Improve match analysis logic and opponent xG data
</commit_message>
<xml_diff>
--- a/data/premier_league_team_tables_home_away.xlsx
+++ b/data/premier_league_team_tables_home_away.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Daniel\Desktop\InStatsWeTrust\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{133C3226-0A5E-4DBD-95C8-CFAF061D331A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{669F083D-39C3-4F70-9B54-E50BD39F7E42}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-32130" yWindow="3600" windowWidth="25875" windowHeight="13455" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="165" yWindow="30" windowWidth="25875" windowHeight="13455" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="HomeTable" sheetId="1" r:id="rId1"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2607" uniqueCount="495">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2607" uniqueCount="477">
   <si>
     <t>Round</t>
   </si>
@@ -1446,60 +1446,6 @@
   </si>
   <si>
     <t>13:35</t>
-  </si>
-  <si>
-    <t>Liverpool FC (L)</t>
-  </si>
-  <si>
-    <t>Arsenal FC</t>
-  </si>
-  <si>
-    <t>Manchester City (M)</t>
-  </si>
-  <si>
-    <t>Newcastle United</t>
-  </si>
-  <si>
-    <t>Chelsea FC</t>
-  </si>
-  <si>
-    <t>Nottingham Forest</t>
-  </si>
-  <si>
-    <t>Brentford FC</t>
-  </si>
-  <si>
-    <t>Fulham FC</t>
-  </si>
-  <si>
-    <t>Brighton &amp; Hove Albion</t>
-  </si>
-  <si>
-    <t>AFC Bournemouth</t>
-  </si>
-  <si>
-    <t>Tottenham Hotspur</t>
-  </si>
-  <si>
-    <t>Manchester United (P)</t>
-  </si>
-  <si>
-    <t>Everton FC</t>
-  </si>
-  <si>
-    <t>West Ham United</t>
-  </si>
-  <si>
-    <t>Wolverhampton Wanderers</t>
-  </si>
-  <si>
-    <t>Leicester City (N)</t>
-  </si>
-  <si>
-    <t>Ipswich Town (N)</t>
-  </si>
-  <si>
-    <t>Southampton FC (N)</t>
   </si>
   <si>
     <t>TEAM</t>
@@ -1882,7 +1828,7 @@
   <dimension ref="A1:J681"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="3" max="3" width="16.140625" customWidth="1"/>
+    <col min="3" max="3" width="26.140625" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="12.42578125" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1891,10 +1837,10 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>494</v>
+        <v>476</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>493</v>
+        <v>475</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>1</v>
@@ -22950,7 +22896,7 @@
         <v>1</v>
       </c>
       <c r="C662" t="s">
-        <v>475</v>
+        <v>19</v>
       </c>
       <c r="D662">
         <v>16</v>
@@ -22982,7 +22928,7 @@
         <v>2</v>
       </c>
       <c r="C663" t="s">
-        <v>476</v>
+        <v>8</v>
       </c>
       <c r="D663">
         <v>16</v>
@@ -23046,7 +22992,7 @@
         <v>4</v>
       </c>
       <c r="C665" t="s">
-        <v>477</v>
+        <v>20</v>
       </c>
       <c r="D665">
         <v>16</v>
@@ -23078,7 +23024,7 @@
         <v>5</v>
       </c>
       <c r="C666" t="s">
-        <v>478</v>
+        <v>11</v>
       </c>
       <c r="D666">
         <v>16</v>
@@ -23110,7 +23056,7 @@
         <v>6</v>
       </c>
       <c r="C667" t="s">
-        <v>479</v>
+        <v>25</v>
       </c>
       <c r="D667">
         <v>16</v>
@@ -23142,7 +23088,7 @@
         <v>7</v>
       </c>
       <c r="C668" t="s">
-        <v>480</v>
+        <v>13</v>
       </c>
       <c r="D668">
         <v>16</v>
@@ -23174,7 +23120,7 @@
         <v>8</v>
       </c>
       <c r="C669" t="s">
-        <v>481</v>
+        <v>9</v>
       </c>
       <c r="D669">
         <v>17</v>
@@ -23206,7 +23152,7 @@
         <v>9</v>
       </c>
       <c r="C670" t="s">
-        <v>482</v>
+        <v>18</v>
       </c>
       <c r="D670">
         <v>17</v>
@@ -23238,7 +23184,7 @@
         <v>10</v>
       </c>
       <c r="C671" t="s">
-        <v>483</v>
+        <v>16</v>
       </c>
       <c r="D671">
         <v>16</v>
@@ -23270,7 +23216,7 @@
         <v>11</v>
       </c>
       <c r="C672" t="s">
-        <v>484</v>
+        <v>14</v>
       </c>
       <c r="D672">
         <v>16</v>
@@ -23302,7 +23248,7 @@
         <v>12</v>
       </c>
       <c r="C673" t="s">
-        <v>485</v>
+        <v>22</v>
       </c>
       <c r="D673">
         <v>17</v>
@@ -23366,7 +23312,7 @@
         <v>14</v>
       </c>
       <c r="C675" t="s">
-        <v>486</v>
+        <v>10</v>
       </c>
       <c r="D675">
         <v>17</v>
@@ -23398,7 +23344,7 @@
         <v>15</v>
       </c>
       <c r="C676" t="s">
-        <v>487</v>
+        <v>27</v>
       </c>
       <c r="D676">
         <v>17</v>
@@ -23430,7 +23376,7 @@
         <v>16</v>
       </c>
       <c r="C677" t="s">
-        <v>488</v>
+        <v>24</v>
       </c>
       <c r="D677">
         <v>17</v>
@@ -23462,7 +23408,7 @@
         <v>17</v>
       </c>
       <c r="C678" t="s">
-        <v>489</v>
+        <v>23</v>
       </c>
       <c r="D678">
         <v>16</v>
@@ -23494,7 +23440,7 @@
         <v>18</v>
       </c>
       <c r="C679" t="s">
-        <v>490</v>
+        <v>12</v>
       </c>
       <c r="D679">
         <v>17</v>
@@ -23526,7 +23472,7 @@
         <v>19</v>
       </c>
       <c r="C680" t="s">
-        <v>491</v>
+        <v>26</v>
       </c>
       <c r="D680">
         <v>17</v>
@@ -23558,7 +23504,7 @@
         <v>20</v>
       </c>
       <c r="C681" t="s">
-        <v>492</v>
+        <v>21</v>
       </c>
       <c r="D681">
         <v>16</v>
@@ -23591,16 +23537,19 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:J681"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="3" max="3" width="71.28515625" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>494</v>
+        <v>476</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>493</v>
+        <v>475</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>1</v>
@@ -44596,7 +44545,7 @@
         <v>1</v>
       </c>
       <c r="C662" t="s">
-        <v>475</v>
+        <v>19</v>
       </c>
       <c r="D662">
         <v>17</v>
@@ -44628,7 +44577,7 @@
         <v>2</v>
       </c>
       <c r="C663" t="s">
-        <v>476</v>
+        <v>8</v>
       </c>
       <c r="D663">
         <v>17</v>
@@ -44660,7 +44609,7 @@
         <v>3</v>
       </c>
       <c r="C664" t="s">
-        <v>480</v>
+        <v>13</v>
       </c>
       <c r="D664">
         <v>17</v>
@@ -44692,7 +44641,7 @@
         <v>4</v>
       </c>
       <c r="C665" t="s">
-        <v>478</v>
+        <v>11</v>
       </c>
       <c r="D665">
         <v>17</v>
@@ -44724,7 +44673,7 @@
         <v>5</v>
       </c>
       <c r="C666" t="s">
-        <v>484</v>
+        <v>14</v>
       </c>
       <c r="D666">
         <v>17</v>
@@ -44756,7 +44705,7 @@
         <v>6</v>
       </c>
       <c r="C667" t="s">
-        <v>477</v>
+        <v>20</v>
       </c>
       <c r="D667">
         <v>17</v>
@@ -44788,7 +44737,7 @@
         <v>7</v>
       </c>
       <c r="C668" t="s">
-        <v>479</v>
+        <v>25</v>
       </c>
       <c r="D668">
         <v>17</v>
@@ -44852,7 +44801,7 @@
         <v>9</v>
       </c>
       <c r="C670" t="s">
-        <v>483</v>
+        <v>16</v>
       </c>
       <c r="D670">
         <v>17</v>
@@ -44916,7 +44865,7 @@
         <v>11</v>
       </c>
       <c r="C672" t="s">
-        <v>482</v>
+        <v>18</v>
       </c>
       <c r="D672">
         <v>16</v>
@@ -44948,7 +44897,7 @@
         <v>12</v>
       </c>
       <c r="C673" t="s">
-        <v>489</v>
+        <v>23</v>
       </c>
       <c r="D673">
         <v>17</v>
@@ -44980,7 +44929,7 @@
         <v>13</v>
       </c>
       <c r="C674" t="s">
-        <v>481</v>
+        <v>9</v>
       </c>
       <c r="D674">
         <v>16</v>
@@ -45012,7 +44961,7 @@
         <v>14</v>
       </c>
       <c r="C675" t="s">
-        <v>487</v>
+        <v>27</v>
       </c>
       <c r="D675">
         <v>16</v>
@@ -45044,7 +44993,7 @@
         <v>15</v>
       </c>
       <c r="C676" t="s">
-        <v>486</v>
+        <v>10</v>
       </c>
       <c r="D676">
         <v>16</v>
@@ -45076,7 +45025,7 @@
         <v>16</v>
       </c>
       <c r="C677" t="s">
-        <v>488</v>
+        <v>24</v>
       </c>
       <c r="D677">
         <v>16</v>
@@ -45108,7 +45057,7 @@
         <v>17</v>
       </c>
       <c r="C678" t="s">
-        <v>485</v>
+        <v>22</v>
       </c>
       <c r="D678">
         <v>16</v>
@@ -45140,7 +45089,7 @@
         <v>18</v>
       </c>
       <c r="C679" t="s">
-        <v>491</v>
+        <v>26</v>
       </c>
       <c r="D679">
         <v>16</v>
@@ -45172,7 +45121,7 @@
         <v>19</v>
       </c>
       <c r="C680" t="s">
-        <v>490</v>
+        <v>12</v>
       </c>
       <c r="D680">
         <v>16</v>
@@ -45204,7 +45153,7 @@
         <v>20</v>
       </c>
       <c r="C681" t="s">
-        <v>492</v>
+        <v>21</v>
       </c>
       <c r="D681">
         <v>17</v>

</xml_diff>

<commit_message>
Add power rating with description
</commit_message>
<xml_diff>
--- a/data/premier_league_team_tables_home_away.xlsx
+++ b/data/premier_league_team_tables_home_away.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Daniel\Desktop\InStatsWeTrust\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{669F083D-39C3-4F70-9B54-E50BD39F7E42}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0F4C7B11-C028-4016-B1BB-14267F999572}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="165" yWindow="30" windowWidth="25875" windowHeight="13455" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-38520" yWindow="-120" windowWidth="38640" windowHeight="21390" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="HomeTable" sheetId="1" r:id="rId1"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2607" uniqueCount="477">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2647" uniqueCount="477">
   <si>
     <t>Round</t>
   </si>
@@ -1825,7 +1825,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:J681"/>
+  <dimension ref="A1:J701"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="3" max="3" width="26.140625" bestFit="1" customWidth="1"/>
@@ -23528,14 +23528,655 @@
         <v>5</v>
       </c>
     </row>
+    <row r="682" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A682">
+        <v>35</v>
+      </c>
+      <c r="B682">
+        <v>1</v>
+      </c>
+      <c r="C682" t="s">
+        <v>19</v>
+      </c>
+      <c r="D682">
+        <v>17</v>
+      </c>
+      <c r="E682">
+        <v>14</v>
+      </c>
+      <c r="F682">
+        <v>2</v>
+      </c>
+      <c r="G682">
+        <v>1</v>
+      </c>
+      <c r="H682" s="3">
+        <v>1.6340277777777779</v>
+      </c>
+      <c r="I682">
+        <v>26</v>
+      </c>
+      <c r="J682">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="683" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A683">
+        <v>35</v>
+      </c>
+      <c r="B683">
+        <v>2</v>
+      </c>
+      <c r="C683" t="s">
+        <v>20</v>
+      </c>
+      <c r="D683">
+        <v>18</v>
+      </c>
+      <c r="E683">
+        <v>12</v>
+      </c>
+      <c r="F683">
+        <v>3</v>
+      </c>
+      <c r="G683">
+        <v>3</v>
+      </c>
+      <c r="H683" s="3">
+        <v>1.6819444444444445</v>
+      </c>
+      <c r="I683">
+        <v>18</v>
+      </c>
+      <c r="J683">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="684" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A684">
+        <v>35</v>
+      </c>
+      <c r="B684">
+        <v>3</v>
+      </c>
+      <c r="C684" t="s">
+        <v>25</v>
+      </c>
+      <c r="D684">
+        <v>18</v>
+      </c>
+      <c r="E684">
+        <v>11</v>
+      </c>
+      <c r="F684">
+        <v>5</v>
+      </c>
+      <c r="G684">
+        <v>2</v>
+      </c>
+      <c r="H684" s="3">
+        <v>1.4291666666666667</v>
+      </c>
+      <c r="I684">
+        <v>16</v>
+      </c>
+      <c r="J684">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="685" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A685">
+        <v>35</v>
+      </c>
+      <c r="B685">
+        <v>4</v>
+      </c>
+      <c r="C685" t="s">
+        <v>15</v>
+      </c>
+      <c r="D685">
+        <v>18</v>
+      </c>
+      <c r="E685">
+        <v>10</v>
+      </c>
+      <c r="F685">
+        <v>7</v>
+      </c>
+      <c r="G685">
+        <v>1</v>
+      </c>
+      <c r="H685" s="3">
+        <v>1.3472222222222223</v>
+      </c>
+      <c r="I685">
+        <v>12</v>
+      </c>
+      <c r="J685">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="686" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A686">
+        <v>35</v>
+      </c>
+      <c r="B686">
+        <v>5</v>
+      </c>
+      <c r="C686" t="s">
+        <v>8</v>
+      </c>
+      <c r="D686">
+        <v>18</v>
+      </c>
+      <c r="E686">
+        <v>10</v>
+      </c>
+      <c r="F686">
+        <v>6</v>
+      </c>
+      <c r="G686">
+        <v>2</v>
+      </c>
+      <c r="H686" s="3">
+        <v>1.4284722222222221</v>
+      </c>
+      <c r="I686">
+        <v>17</v>
+      </c>
+      <c r="J686">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="687" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A687">
+        <v>35</v>
+      </c>
+      <c r="B687">
+        <v>6</v>
+      </c>
+      <c r="C687" t="s">
+        <v>11</v>
+      </c>
+      <c r="D687">
+        <v>17</v>
+      </c>
+      <c r="E687">
+        <v>11</v>
+      </c>
+      <c r="F687">
+        <v>2</v>
+      </c>
+      <c r="G687">
+        <v>4</v>
+      </c>
+      <c r="H687" s="3">
+        <v>1.5965277777777778</v>
+      </c>
+      <c r="I687">
+        <v>19</v>
+      </c>
+      <c r="J687">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="688" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A688">
+        <v>35</v>
+      </c>
+      <c r="B688">
+        <v>7</v>
+      </c>
+      <c r="C688" t="s">
+        <v>13</v>
+      </c>
+      <c r="D688">
+        <v>17</v>
+      </c>
+      <c r="E688">
+        <v>9</v>
+      </c>
+      <c r="F688">
+        <v>4</v>
+      </c>
+      <c r="G688">
+        <v>4</v>
+      </c>
+      <c r="H688" s="3">
+        <v>1.0090277777777779</v>
+      </c>
+      <c r="I688">
+        <v>11</v>
+      </c>
+      <c r="J688">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="689" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A689">
+        <v>35</v>
+      </c>
+      <c r="B689">
+        <v>8</v>
+      </c>
+      <c r="C689" t="s">
+        <v>9</v>
+      </c>
+      <c r="D689">
+        <v>18</v>
+      </c>
+      <c r="E689">
+        <v>9</v>
+      </c>
+      <c r="F689">
+        <v>4</v>
+      </c>
+      <c r="G689">
+        <v>5</v>
+      </c>
+      <c r="H689" s="3">
+        <v>1.6055555555555556</v>
+      </c>
+      <c r="I689">
+        <v>6</v>
+      </c>
+      <c r="J689">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="690" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A690">
+        <v>35</v>
+      </c>
+      <c r="B690">
+        <v>9</v>
+      </c>
+      <c r="C690" t="s">
+        <v>16</v>
+      </c>
+      <c r="D690">
+        <v>18</v>
+      </c>
+      <c r="E690">
+        <v>7</v>
+      </c>
+      <c r="F690">
+        <v>8</v>
+      </c>
+      <c r="G690">
+        <v>3</v>
+      </c>
+      <c r="H690" s="3">
+        <v>1.1416666666666666</v>
+      </c>
+      <c r="I690">
+        <v>3</v>
+      </c>
+      <c r="J690">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="691" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A691">
+        <v>35</v>
+      </c>
+      <c r="B691">
+        <v>10</v>
+      </c>
+      <c r="C691" t="s">
+        <v>18</v>
+      </c>
+      <c r="D691">
+        <v>17</v>
+      </c>
+      <c r="E691">
+        <v>7</v>
+      </c>
+      <c r="F691">
+        <v>5</v>
+      </c>
+      <c r="G691">
+        <v>5</v>
+      </c>
+      <c r="H691" s="3">
+        <v>1.1006944444444444</v>
+      </c>
+      <c r="I691">
+        <v>1</v>
+      </c>
+      <c r="J691">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="692" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A692">
+        <v>35</v>
+      </c>
+      <c r="B692">
+        <v>11</v>
+      </c>
+      <c r="C692" t="s">
+        <v>14</v>
+      </c>
+      <c r="D692">
+        <v>17</v>
+      </c>
+      <c r="E692">
+        <v>7</v>
+      </c>
+      <c r="F692">
+        <v>4</v>
+      </c>
+      <c r="G692">
+        <v>6</v>
+      </c>
+      <c r="H692" s="4">
+        <v>0.88541666666666663</v>
+      </c>
+      <c r="I692">
+        <v>6</v>
+      </c>
+      <c r="J692">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="693" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A693">
+        <v>35</v>
+      </c>
+      <c r="B693">
+        <v>12</v>
+      </c>
+      <c r="C693" t="s">
+        <v>17</v>
+      </c>
+      <c r="D693">
+        <v>18</v>
+      </c>
+      <c r="E693">
+        <v>5</v>
+      </c>
+      <c r="F693">
+        <v>7</v>
+      </c>
+      <c r="G693">
+        <v>6</v>
+      </c>
+      <c r="H693" s="4">
+        <v>0.85</v>
+      </c>
+      <c r="I693">
+        <v>-4</v>
+      </c>
+      <c r="J693">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="694" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A694">
+        <v>35</v>
+      </c>
+      <c r="B694">
+        <v>13</v>
+      </c>
+      <c r="C694" t="s">
+        <v>22</v>
+      </c>
+      <c r="D694">
+        <v>17</v>
+      </c>
+      <c r="E694">
+        <v>6</v>
+      </c>
+      <c r="F694">
+        <v>3</v>
+      </c>
+      <c r="G694">
+        <v>8</v>
+      </c>
+      <c r="H694" s="3">
+        <v>1.4368055555555554</v>
+      </c>
+      <c r="I694">
+        <v>5</v>
+      </c>
+      <c r="J694">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="695" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A695">
+        <v>35</v>
+      </c>
+      <c r="B695">
+        <v>14</v>
+      </c>
+      <c r="C695" t="s">
+        <v>27</v>
+      </c>
+      <c r="D695">
+        <v>18</v>
+      </c>
+      <c r="E695">
+        <v>4</v>
+      </c>
+      <c r="F695">
+        <v>9</v>
+      </c>
+      <c r="G695">
+        <v>5</v>
+      </c>
+      <c r="H695" s="3">
+        <v>1.0159722222222223</v>
+      </c>
+      <c r="I695">
+        <v>1</v>
+      </c>
+      <c r="J695">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="696" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A696">
+        <v>35</v>
+      </c>
+      <c r="B696">
+        <v>15</v>
+      </c>
+      <c r="C696" t="s">
+        <v>10</v>
+      </c>
+      <c r="D696">
+        <v>17</v>
+      </c>
+      <c r="E696">
+        <v>6</v>
+      </c>
+      <c r="F696">
+        <v>3</v>
+      </c>
+      <c r="G696">
+        <v>8</v>
+      </c>
+      <c r="H696" s="4">
+        <v>0.8930555555555556</v>
+      </c>
+      <c r="I696">
+        <v>-5</v>
+      </c>
+      <c r="J696">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="697" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A697">
+        <v>35</v>
+      </c>
+      <c r="B697">
+        <v>16</v>
+      </c>
+      <c r="C697" t="s">
+        <v>23</v>
+      </c>
+      <c r="D697">
+        <v>17</v>
+      </c>
+      <c r="E697">
+        <v>6</v>
+      </c>
+      <c r="F697">
+        <v>2</v>
+      </c>
+      <c r="G697">
+        <v>9</v>
+      </c>
+      <c r="H697" s="3">
+        <v>1.1034722222222222</v>
+      </c>
+      <c r="I697">
+        <v>-3</v>
+      </c>
+      <c r="J697">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="698" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A698">
+        <v>35</v>
+      </c>
+      <c r="B698">
+        <v>17</v>
+      </c>
+      <c r="C698" t="s">
+        <v>24</v>
+      </c>
+      <c r="D698">
+        <v>18</v>
+      </c>
+      <c r="E698">
+        <v>5</v>
+      </c>
+      <c r="F698">
+        <v>5</v>
+      </c>
+      <c r="G698">
+        <v>8</v>
+      </c>
+      <c r="H698" s="4">
+        <v>0.93888888888888888</v>
+      </c>
+      <c r="I698">
+        <v>-10</v>
+      </c>
+      <c r="J698">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="699" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A699">
+        <v>35</v>
+      </c>
+      <c r="B699">
+        <v>18</v>
+      </c>
+      <c r="C699" t="s">
+        <v>12</v>
+      </c>
+      <c r="D699">
+        <v>18</v>
+      </c>
+      <c r="E699">
+        <v>3</v>
+      </c>
+      <c r="F699">
+        <v>3</v>
+      </c>
+      <c r="G699">
+        <v>12</v>
+      </c>
+      <c r="H699" s="4">
+        <v>0.56527777777777777</v>
+      </c>
+      <c r="I699">
+        <v>-21</v>
+      </c>
+      <c r="J699">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="700" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A700">
+        <v>35</v>
+      </c>
+      <c r="B700">
+        <v>19</v>
+      </c>
+      <c r="C700" t="s">
+        <v>26</v>
+      </c>
+      <c r="D700">
+        <v>17</v>
+      </c>
+      <c r="E700">
+        <v>1</v>
+      </c>
+      <c r="F700">
+        <v>4</v>
+      </c>
+      <c r="G700">
+        <v>12</v>
+      </c>
+      <c r="H700" s="4">
+        <v>0.56944444444444442</v>
+      </c>
+      <c r="I700">
+        <v>-27</v>
+      </c>
+      <c r="J700">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="701" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A701">
+        <v>35</v>
+      </c>
+      <c r="B701">
+        <v>20</v>
+      </c>
+      <c r="C701" t="s">
+        <v>21</v>
+      </c>
+      <c r="D701">
+        <v>17</v>
+      </c>
+      <c r="E701">
+        <v>1</v>
+      </c>
+      <c r="F701">
+        <v>2</v>
+      </c>
+      <c r="G701">
+        <v>14</v>
+      </c>
+      <c r="H701" s="4">
+        <v>0.53125</v>
+      </c>
+      <c r="I701">
+        <v>-33</v>
+      </c>
+      <c r="J701">
+        <v>5</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:J681"/>
+  <dimension ref="A1:J701"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="3" max="3" width="71.28515625" customWidth="1"/>
@@ -45177,6 +45818,646 @@
         <v>6</v>
       </c>
     </row>
+    <row r="682" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A682">
+        <v>35</v>
+      </c>
+      <c r="B682">
+        <v>1</v>
+      </c>
+      <c r="C682" t="s">
+        <v>19</v>
+      </c>
+      <c r="D682">
+        <v>18</v>
+      </c>
+      <c r="E682">
+        <v>11</v>
+      </c>
+      <c r="F682">
+        <v>5</v>
+      </c>
+      <c r="G682">
+        <v>2</v>
+      </c>
+      <c r="H682" s="3">
+        <v>1.7652777777777777</v>
+      </c>
+      <c r="I682">
+        <v>20</v>
+      </c>
+      <c r="J682">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="683" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A683">
+        <v>35</v>
+      </c>
+      <c r="B683">
+        <v>2</v>
+      </c>
+      <c r="C683" t="s">
+        <v>8</v>
+      </c>
+      <c r="D683">
+        <v>17</v>
+      </c>
+      <c r="E683">
+        <v>8</v>
+      </c>
+      <c r="F683">
+        <v>7</v>
+      </c>
+      <c r="G683">
+        <v>2</v>
+      </c>
+      <c r="H683" s="3">
+        <v>1.2597222222222222</v>
+      </c>
+      <c r="I683">
+        <v>16</v>
+      </c>
+      <c r="J683">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="684" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A684">
+        <v>35</v>
+      </c>
+      <c r="B684">
+        <v>3</v>
+      </c>
+      <c r="C684" t="s">
+        <v>13</v>
+      </c>
+      <c r="D684">
+        <v>18</v>
+      </c>
+      <c r="E684">
+        <v>9</v>
+      </c>
+      <c r="F684">
+        <v>3</v>
+      </c>
+      <c r="G684">
+        <v>6</v>
+      </c>
+      <c r="H684" s="3">
+        <v>1.2701388888888889</v>
+      </c>
+      <c r="I684">
+        <v>1</v>
+      </c>
+      <c r="J684">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="685" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A685">
+        <v>35</v>
+      </c>
+      <c r="B685">
+        <v>4</v>
+      </c>
+      <c r="C685" t="s">
+        <v>14</v>
+      </c>
+      <c r="D685">
+        <v>18</v>
+      </c>
+      <c r="E685">
+        <v>7</v>
+      </c>
+      <c r="F685">
+        <v>7</v>
+      </c>
+      <c r="G685">
+        <v>4</v>
+      </c>
+      <c r="H685" s="3">
+        <v>1.4354166666666666</v>
+      </c>
+      <c r="I685">
+        <v>7</v>
+      </c>
+      <c r="J685">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="686" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A686">
+        <v>35</v>
+      </c>
+      <c r="B686">
+        <v>5</v>
+      </c>
+      <c r="C686" t="s">
+        <v>11</v>
+      </c>
+      <c r="D686">
+        <v>18</v>
+      </c>
+      <c r="E686">
+        <v>8</v>
+      </c>
+      <c r="F686">
+        <v>4</v>
+      </c>
+      <c r="G686">
+        <v>6</v>
+      </c>
+      <c r="H686" s="3">
+        <v>1.1847222222222222</v>
+      </c>
+      <c r="I686">
+        <v>2</v>
+      </c>
+      <c r="J686">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="687" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A687">
+        <v>35</v>
+      </c>
+      <c r="B687">
+        <v>6</v>
+      </c>
+      <c r="C687" t="s">
+        <v>20</v>
+      </c>
+      <c r="D687">
+        <v>17</v>
+      </c>
+      <c r="E687">
+        <v>7</v>
+      </c>
+      <c r="F687">
+        <v>4</v>
+      </c>
+      <c r="G687">
+        <v>6</v>
+      </c>
+      <c r="H687" s="3">
+        <v>1.1395833333333334</v>
+      </c>
+      <c r="I687">
+        <v>6</v>
+      </c>
+      <c r="J687">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="688" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A688">
+        <v>35</v>
+      </c>
+      <c r="B688">
+        <v>7</v>
+      </c>
+      <c r="C688" t="s">
+        <v>25</v>
+      </c>
+      <c r="D688">
+        <v>17</v>
+      </c>
+      <c r="E688">
+        <v>7</v>
+      </c>
+      <c r="F688">
+        <v>4</v>
+      </c>
+      <c r="G688">
+        <v>6</v>
+      </c>
+      <c r="H688" s="3">
+        <v>1.1826388888888888</v>
+      </c>
+      <c r="I688">
+        <v>5</v>
+      </c>
+      <c r="J688">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="689" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A689">
+        <v>35</v>
+      </c>
+      <c r="B689">
+        <v>8</v>
+      </c>
+      <c r="C689" t="s">
+        <v>18</v>
+      </c>
+      <c r="D689">
+        <v>18</v>
+      </c>
+      <c r="E689">
+        <v>7</v>
+      </c>
+      <c r="F689">
+        <v>4</v>
+      </c>
+      <c r="G689">
+        <v>7</v>
+      </c>
+      <c r="H689" s="3">
+        <v>1.0152777777777777</v>
+      </c>
+      <c r="I689">
+        <v>2</v>
+      </c>
+      <c r="J689">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="690" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A690">
+        <v>35</v>
+      </c>
+      <c r="B690">
+        <v>9</v>
+      </c>
+      <c r="C690" t="s">
+        <v>17</v>
+      </c>
+      <c r="D690">
+        <v>17</v>
+      </c>
+      <c r="E690">
+        <v>6</v>
+      </c>
+      <c r="F690">
+        <v>6</v>
+      </c>
+      <c r="G690">
+        <v>5</v>
+      </c>
+      <c r="H690" s="3">
+        <v>1.0166666666666666</v>
+      </c>
+      <c r="I690">
+        <v>0</v>
+      </c>
+      <c r="J690">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="691" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A691">
+        <v>35</v>
+      </c>
+      <c r="B691">
+        <v>10</v>
+      </c>
+      <c r="C691" t="s">
+        <v>16</v>
+      </c>
+      <c r="D691">
+        <v>17</v>
+      </c>
+      <c r="E691">
+        <v>6</v>
+      </c>
+      <c r="F691">
+        <v>5</v>
+      </c>
+      <c r="G691">
+        <v>6</v>
+      </c>
+      <c r="H691" s="3">
+        <v>1.2722222222222221</v>
+      </c>
+      <c r="I691">
+        <v>-2</v>
+      </c>
+      <c r="J691">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="692" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A692">
+        <v>35</v>
+      </c>
+      <c r="B692">
+        <v>11</v>
+      </c>
+      <c r="C692" t="s">
+        <v>15</v>
+      </c>
+      <c r="D692">
+        <v>17</v>
+      </c>
+      <c r="E692">
+        <v>7</v>
+      </c>
+      <c r="F692">
+        <v>2</v>
+      </c>
+      <c r="G692">
+        <v>8</v>
+      </c>
+      <c r="H692" s="4">
+        <v>0.97847222222222219</v>
+      </c>
+      <c r="I692">
+        <v>-6</v>
+      </c>
+      <c r="J692">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="693" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A693">
+        <v>35</v>
+      </c>
+      <c r="B693">
+        <v>12</v>
+      </c>
+      <c r="C693" t="s">
+        <v>9</v>
+      </c>
+      <c r="D693">
+        <v>17</v>
+      </c>
+      <c r="E693">
+        <v>6</v>
+      </c>
+      <c r="F693">
+        <v>3</v>
+      </c>
+      <c r="G693">
+        <v>8</v>
+      </c>
+      <c r="H693" s="3">
+        <v>1.0145833333333334</v>
+      </c>
+      <c r="I693">
+        <v>3</v>
+      </c>
+      <c r="J693">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="694" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A694">
+        <v>35</v>
+      </c>
+      <c r="B694">
+        <v>13</v>
+      </c>
+      <c r="C694" t="s">
+        <v>23</v>
+      </c>
+      <c r="D694">
+        <v>18</v>
+      </c>
+      <c r="E694">
+        <v>6</v>
+      </c>
+      <c r="F694">
+        <v>3</v>
+      </c>
+      <c r="G694">
+        <v>9</v>
+      </c>
+      <c r="H694" s="3">
+        <v>1.0645833333333334</v>
+      </c>
+      <c r="I694">
+        <v>-8</v>
+      </c>
+      <c r="J694">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="695" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A695">
+        <v>35</v>
+      </c>
+      <c r="B695">
+        <v>14</v>
+      </c>
+      <c r="C695" t="s">
+        <v>10</v>
+      </c>
+      <c r="D695">
+        <v>18</v>
+      </c>
+      <c r="E695">
+        <v>4</v>
+      </c>
+      <c r="F695">
+        <v>6</v>
+      </c>
+      <c r="G695">
+        <v>8</v>
+      </c>
+      <c r="H695" s="4">
+        <v>0.89236111111111116</v>
+      </c>
+      <c r="I695">
+        <v>-4</v>
+      </c>
+      <c r="J695">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="696" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A696">
+        <v>35</v>
+      </c>
+      <c r="B696">
+        <v>15</v>
+      </c>
+      <c r="C696" t="s">
+        <v>27</v>
+      </c>
+      <c r="D696">
+        <v>17</v>
+      </c>
+      <c r="E696">
+        <v>4</v>
+      </c>
+      <c r="F696">
+        <v>6</v>
+      </c>
+      <c r="G696">
+        <v>7</v>
+      </c>
+      <c r="H696" s="4">
+        <v>0.51388888888888884</v>
+      </c>
+      <c r="I696">
+        <v>-8</v>
+      </c>
+      <c r="J696">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="697" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A697">
+        <v>35</v>
+      </c>
+      <c r="B697">
+        <v>16</v>
+      </c>
+      <c r="C697" t="s">
+        <v>22</v>
+      </c>
+      <c r="D697">
+        <v>18</v>
+      </c>
+      <c r="E697">
+        <v>5</v>
+      </c>
+      <c r="F697">
+        <v>2</v>
+      </c>
+      <c r="G697">
+        <v>11</v>
+      </c>
+      <c r="H697" s="3">
+        <v>1.2277777777777779</v>
+      </c>
+      <c r="I697">
+        <v>1</v>
+      </c>
+      <c r="J697">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="698" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A698">
+        <v>35</v>
+      </c>
+      <c r="B698">
+        <v>17</v>
+      </c>
+      <c r="C698" t="s">
+        <v>24</v>
+      </c>
+      <c r="D698">
+        <v>17</v>
+      </c>
+      <c r="E698">
+        <v>4</v>
+      </c>
+      <c r="F698">
+        <v>5</v>
+      </c>
+      <c r="G698">
+        <v>8</v>
+      </c>
+      <c r="H698" s="4">
+        <v>0.76875000000000004</v>
+      </c>
+      <c r="I698">
+        <v>-9</v>
+      </c>
+      <c r="J698">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="699" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A699">
+        <v>35</v>
+      </c>
+      <c r="B699">
+        <v>18</v>
+      </c>
+      <c r="C699" t="s">
+        <v>26</v>
+      </c>
+      <c r="D699">
+        <v>18</v>
+      </c>
+      <c r="E699">
+        <v>3</v>
+      </c>
+      <c r="F699">
+        <v>6</v>
+      </c>
+      <c r="G699">
+        <v>9</v>
+      </c>
+      <c r="H699" s="4">
+        <v>0.94166666666666665</v>
+      </c>
+      <c r="I699">
+        <v>-14</v>
+      </c>
+      <c r="J699">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="700" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A700">
+        <v>35</v>
+      </c>
+      <c r="B700">
+        <v>19</v>
+      </c>
+      <c r="C700" t="s">
+        <v>12</v>
+      </c>
+      <c r="D700">
+        <v>17</v>
+      </c>
+      <c r="E700">
+        <v>2</v>
+      </c>
+      <c r="F700">
+        <v>3</v>
+      </c>
+      <c r="G700">
+        <v>12</v>
+      </c>
+      <c r="H700" s="4">
+        <v>0.6958333333333333</v>
+      </c>
+      <c r="I700">
+        <v>-26</v>
+      </c>
+      <c r="J700">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="701" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A701">
+        <v>35</v>
+      </c>
+      <c r="B701">
+        <v>20</v>
+      </c>
+      <c r="C701" t="s">
+        <v>21</v>
+      </c>
+      <c r="D701">
+        <v>18</v>
+      </c>
+      <c r="E701">
+        <v>1</v>
+      </c>
+      <c r="F701">
+        <v>3</v>
+      </c>
+      <c r="G701">
+        <v>14</v>
+      </c>
+      <c r="H701" s="4">
+        <v>0.56736111111111109</v>
+      </c>
+      <c r="I701">
+        <v>-24</v>
+      </c>
+      <c r="J701">
+        <v>6</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>